<commit_message>
more time depedent dataset and logic
</commit_message>
<xml_diff>
--- a/data/facility.xlsx
+++ b/data/facility.xlsx
@@ -1,26 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29530"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Codes\Python\PyCharm Projects\private-credit-performance\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C68510C-0D24-4D24-90F5-9C436E56FB80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>date</t>
   </si>
@@ -42,28 +36,15 @@
   <si>
     <t>cost_of_funds</t>
   </si>
-  <si>
-    <t>2024-09-30</t>
-  </si>
-  <si>
-    <t>2024-10-31</t>
-  </si>
-  <si>
-    <t>2024-11-30</t>
-  </si>
-  <si>
-    <t>2024-12-31</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -73,13 +54,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -119,38 +93,28 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -188,7 +152,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -222,7 +186,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -257,10 +220,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -433,19 +395,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.5703125" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -468,96 +422,280 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="2">
-        <v>60000000</v>
-      </c>
-      <c r="C2" s="2">
+    <row r="2" spans="1:7">
+      <c r="A2" s="2">
+        <v>45322</v>
+      </c>
+      <c r="B2">
+        <v>51879950</v>
+      </c>
+      <c r="C2">
         <v>90000000</v>
       </c>
       <c r="D2">
         <v>0.7</v>
       </c>
       <c r="E2">
-        <v>0.18</v>
+        <v>0.2</v>
       </c>
       <c r="F2">
-        <v>0.22</v>
+        <v>0.24</v>
       </c>
       <c r="G2">
-        <v>4.4999999999999998E-2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="2">
-        <v>64000000</v>
-      </c>
-      <c r="C3" s="2">
+        <v>0.045</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="2">
+        <v>45351</v>
+      </c>
+      <c r="B3">
+        <v>53962265</v>
+      </c>
+      <c r="C3">
         <v>90000000</v>
       </c>
       <c r="D3">
         <v>0.7</v>
       </c>
       <c r="E3">
+        <v>0.193</v>
+      </c>
+      <c r="F3">
+        <v>0.232</v>
+      </c>
+      <c r="G3">
+        <v>0.04527272727272727</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="2">
+        <v>45382</v>
+      </c>
+      <c r="B4">
+        <v>56186235.5</v>
+      </c>
+      <c r="C4">
+        <v>90000000</v>
+      </c>
+      <c r="D4">
+        <v>0.7</v>
+      </c>
+      <c r="E4">
+        <v>0.186</v>
+      </c>
+      <c r="F4">
+        <v>0.224</v>
+      </c>
+      <c r="G4">
+        <v>0.04554545454545454</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="2">
+        <v>45412</v>
+      </c>
+      <c r="B5">
+        <v>57789364.84999999</v>
+      </c>
+      <c r="C5">
+        <v>90000000</v>
+      </c>
+      <c r="D5">
+        <v>0.7</v>
+      </c>
+      <c r="E5">
+        <v>0.179</v>
+      </c>
+      <c r="F5">
+        <v>0.216</v>
+      </c>
+      <c r="G5">
+        <v>0.04581818181818181</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="2">
+        <v>45443</v>
+      </c>
+      <c r="B6">
+        <v>59317905.395</v>
+      </c>
+      <c r="C6">
+        <v>90000000</v>
+      </c>
+      <c r="D6">
+        <v>0.7</v>
+      </c>
+      <c r="E6">
+        <v>0.172</v>
+      </c>
+      <c r="F6">
+        <v>0.208</v>
+      </c>
+      <c r="G6">
+        <v>0.04609090909090909</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="2">
+        <v>45473</v>
+      </c>
+      <c r="B7">
+        <v>60277309.77649999</v>
+      </c>
+      <c r="C7">
+        <v>90000000</v>
+      </c>
+      <c r="D7">
+        <v>0.7</v>
+      </c>
+      <c r="E7">
+        <v>0.165</v>
+      </c>
+      <c r="F7">
+        <v>0.2</v>
+      </c>
+      <c r="G7">
+        <v>0.04636363636363636</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="2">
+        <v>45504</v>
+      </c>
+      <c r="B8">
+        <v>60645718.84355</v>
+      </c>
+      <c r="C8">
+        <v>90000000</v>
+      </c>
+      <c r="D8">
+        <v>0.7</v>
+      </c>
+      <c r="E8">
+        <v>0.158</v>
+      </c>
+      <c r="F8">
+        <v>0.192</v>
+      </c>
+      <c r="G8">
+        <v>0.04663636363636364</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="2">
+        <v>45535</v>
+      </c>
+      <c r="B9">
+        <v>60718241.19048499</v>
+      </c>
+      <c r="C9">
+        <v>90000000</v>
+      </c>
+      <c r="D9">
+        <v>0.7</v>
+      </c>
+      <c r="E9">
+        <v>0.151</v>
+      </c>
+      <c r="F9">
+        <v>0.184</v>
+      </c>
+      <c r="G9">
+        <v>0.04690909090909091</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="2">
+        <v>45565</v>
+      </c>
+      <c r="B10">
+        <v>60353872.83333949</v>
+      </c>
+      <c r="C10">
+        <v>90000000</v>
+      </c>
+      <c r="D10">
+        <v>0.7</v>
+      </c>
+      <c r="E10">
+        <v>0.144</v>
+      </c>
+      <c r="F10">
+        <v>0.176</v>
+      </c>
+      <c r="G10">
+        <v>0.04718181818181818</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="2">
+        <v>45596</v>
+      </c>
+      <c r="B11">
+        <v>59742468.98333764</v>
+      </c>
+      <c r="C11">
+        <v>90000000</v>
+      </c>
+      <c r="D11">
+        <v>0.7</v>
+      </c>
+      <c r="E11">
+        <v>0.137</v>
+      </c>
+      <c r="F11">
+        <v>0.168</v>
+      </c>
+      <c r="G11">
+        <v>0.04745454545454545</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="2">
+        <v>45626</v>
+      </c>
+      <c r="B12">
+        <v>59138140.28833634</v>
+      </c>
+      <c r="C12">
+        <v>90000000</v>
+      </c>
+      <c r="D12">
+        <v>0.7</v>
+      </c>
+      <c r="E12">
+        <v>0.13</v>
+      </c>
+      <c r="F12">
         <v>0.16</v>
       </c>
-      <c r="F3">
-        <v>0.2</v>
-      </c>
-      <c r="G3">
-        <v>4.5999999999999999E-2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="2">
-        <v>68000000</v>
-      </c>
-      <c r="C4" s="2">
-        <v>90000000</v>
-      </c>
-      <c r="D4">
-        <v>0.7</v>
-      </c>
-      <c r="E4">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="F4">
-        <v>0.18</v>
-      </c>
-      <c r="G4">
-        <v>4.7E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="2">
-        <v>72000000</v>
-      </c>
-      <c r="C5" s="2">
-        <v>90000000</v>
-      </c>
-      <c r="D5">
-        <v>0.7</v>
-      </c>
-      <c r="E5">
-        <v>0.12</v>
-      </c>
-      <c r="F5">
-        <v>0.15</v>
-      </c>
-      <c r="G5">
-        <v>4.8000000000000001E-2</v>
+      <c r="G12">
+        <v>0.04772727272727272</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="2">
+        <v>45657</v>
+      </c>
+      <c r="B13">
+        <v>58448764.20183544</v>
+      </c>
+      <c r="C13">
+        <v>90000000</v>
+      </c>
+      <c r="D13">
+        <v>0.7</v>
+      </c>
+      <c r="E13">
+        <v>0.123</v>
+      </c>
+      <c r="F13">
+        <v>0.152</v>
+      </c>
+      <c r="G13">
+        <v>0.048</v>
       </c>
     </row>
   </sheetData>

</xml_diff>